<commit_message>
feat(nomenclature) : generate files with new values (CISU v2.3)
</commit_message>
<xml_diff>
--- a/nomenclature_parser/in/Nomenclatures RC-EDA et messages RS.xlsx
+++ b/nomenclature_parser/in/Nomenclatures RC-EDA et messages RS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SAMU-Hub\SAMU-Hub-Modeles\nomenclature_parser\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB098801-D6FB-4E33-BBA4-0A1286AABEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9CA1DD-F911-4A73-86D7-7B7227BE85AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="859" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="859" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="#Sommaire" sheetId="1" r:id="rId1"/>
@@ -12725,7 +12725,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R224"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.8"/>
   <cols>
@@ -12805,7 +12804,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="3" spans="1:18" ht="15" customHeight="1">
       <c r="A3" s="78" t="s">
         <v>334</v>
       </c>
@@ -12848,7 +12847,7 @@
       <c r="Q3" s="10"/>
       <c r="R3" s="10"/>
     </row>
-    <row r="4" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="4" spans="1:18" ht="15" customHeight="1">
       <c r="A4" s="70" t="s">
         <v>339</v>
       </c>
@@ -12889,7 +12888,7 @@
       <c r="Q4" s="10"/>
       <c r="R4" s="10"/>
     </row>
-    <row r="5" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="5" spans="1:18" ht="15" customHeight="1">
       <c r="A5" s="70" t="s">
         <v>341</v>
       </c>
@@ -13112,7 +13111,7 @@
       <c r="Q9" s="10"/>
       <c r="R9" s="10"/>
     </row>
-    <row r="10" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="10" spans="1:18" ht="15" customHeight="1">
       <c r="A10" s="70" t="s">
         <v>351</v>
       </c>
@@ -13155,7 +13154,7 @@
       <c r="Q10" s="10"/>
       <c r="R10" s="10"/>
     </row>
-    <row r="11" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="11" spans="1:18" ht="15" customHeight="1">
       <c r="A11" s="77" t="s">
         <v>353</v>
       </c>
@@ -13196,7 +13195,7 @@
       <c r="Q11" s="10"/>
       <c r="R11" s="10"/>
     </row>
-    <row r="12" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="12" spans="1:18" ht="15" customHeight="1">
       <c r="A12" s="70" t="s">
         <v>355</v>
       </c>
@@ -13237,7 +13236,7 @@
       <c r="Q12" s="10"/>
       <c r="R12" s="10"/>
     </row>
-    <row r="13" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="13" spans="1:18" ht="15" customHeight="1">
       <c r="A13" s="70" t="s">
         <v>357</v>
       </c>
@@ -13278,7 +13277,7 @@
       <c r="Q13" s="10"/>
       <c r="R13" s="10"/>
     </row>
-    <row r="14" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="14" spans="1:18" ht="15" customHeight="1">
       <c r="A14" s="70" t="s">
         <v>359</v>
       </c>
@@ -13321,7 +13320,7 @@
       <c r="Q14" s="10"/>
       <c r="R14" s="10"/>
     </row>
-    <row r="15" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="15" spans="1:18" ht="15" customHeight="1">
       <c r="A15" s="70" t="s">
         <v>361</v>
       </c>
@@ -13366,7 +13365,7 @@
       <c r="Q15" s="10"/>
       <c r="R15" s="10"/>
     </row>
-    <row r="16" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="16" spans="1:18" ht="15" customHeight="1">
       <c r="A16" s="70" t="s">
         <v>364</v>
       </c>
@@ -13409,7 +13408,7 @@
       <c r="Q16" s="10"/>
       <c r="R16" s="10"/>
     </row>
-    <row r="17" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="17" spans="1:18" ht="15" customHeight="1">
       <c r="A17" s="70" t="s">
         <v>366</v>
       </c>
@@ -13454,7 +13453,7 @@
       <c r="Q17" s="10"/>
       <c r="R17" s="10"/>
     </row>
-    <row r="18" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="18" spans="1:18" ht="15" customHeight="1">
       <c r="A18" s="70" t="s">
         <v>368</v>
       </c>
@@ -13499,7 +13498,7 @@
       <c r="Q18" s="10"/>
       <c r="R18" s="10"/>
     </row>
-    <row r="19" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="19" spans="1:18" ht="15" customHeight="1">
       <c r="A19" s="77" t="s">
         <v>370</v>
       </c>
@@ -13540,7 +13539,7 @@
       <c r="Q19" s="10"/>
       <c r="R19" s="10"/>
     </row>
-    <row r="20" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="20" spans="1:18" ht="15" customHeight="1">
       <c r="A20" s="70" t="s">
         <v>373</v>
       </c>
@@ -13583,7 +13582,7 @@
       <c r="Q20" s="10"/>
       <c r="R20" s="10"/>
     </row>
-    <row r="21" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="21" spans="1:18" ht="15" customHeight="1">
       <c r="A21" s="70" t="s">
         <v>375</v>
       </c>
@@ -13628,7 +13627,7 @@
       <c r="Q21" s="10"/>
       <c r="R21" s="10"/>
     </row>
-    <row r="22" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="22" spans="1:18" ht="15" customHeight="1">
       <c r="A22" s="71" t="s">
         <v>377</v>
       </c>
@@ -13668,7 +13667,7 @@
       <c r="Q22" s="10"/>
       <c r="R22" s="10"/>
     </row>
-    <row r="23" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="23" spans="1:18" ht="15" customHeight="1">
       <c r="A23" s="70" t="s">
         <v>380</v>
       </c>
@@ -13711,7 +13710,7 @@
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
     </row>
-    <row r="24" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="24" spans="1:18" ht="15" customHeight="1">
       <c r="A24" s="70" t="s">
         <v>382</v>
       </c>
@@ -13754,7 +13753,7 @@
       <c r="Q24" s="10"/>
       <c r="R24" s="10"/>
     </row>
-    <row r="25" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="25" spans="1:18" ht="15" customHeight="1">
       <c r="A25" s="71" t="s">
         <v>384</v>
       </c>
@@ -13799,7 +13798,7 @@
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
     </row>
-    <row r="26" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="26" spans="1:18" ht="15" customHeight="1">
       <c r="A26" s="70" t="s">
         <v>387</v>
       </c>
@@ -13848,7 +13847,7 @@
       <c r="Q26" s="10"/>
       <c r="R26" s="10"/>
     </row>
-    <row r="27" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="27" spans="1:18" ht="15" customHeight="1">
       <c r="A27" s="71" t="s">
         <v>389</v>
       </c>
@@ -13891,7 +13890,7 @@
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
     </row>
-    <row r="28" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="28" spans="1:18" ht="15" customHeight="1">
       <c r="A28" s="71" t="s">
         <v>392</v>
       </c>
@@ -13936,7 +13935,7 @@
       <c r="Q28" s="10"/>
       <c r="R28" s="10"/>
     </row>
-    <row r="29" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="29" spans="1:18" ht="15" customHeight="1">
       <c r="A29" s="70" t="s">
         <v>395</v>
       </c>
@@ -13979,7 +13978,7 @@
       <c r="Q29" s="10"/>
       <c r="R29" s="10"/>
     </row>
-    <row r="30" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="30" spans="1:18" ht="15" customHeight="1">
       <c r="A30" s="70" t="s">
         <v>398</v>
       </c>
@@ -14027,7 +14026,7 @@
       <c r="Q30" s="10"/>
       <c r="R30" s="10"/>
     </row>
-    <row r="31" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="31" spans="1:18" ht="15" customHeight="1">
       <c r="A31" s="71" t="s">
         <v>401</v>
       </c>
@@ -14072,7 +14071,7 @@
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
     </row>
-    <row r="32" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="32" spans="1:18" ht="15" customHeight="1">
       <c r="A32" s="70" t="s">
         <v>403</v>
       </c>
@@ -14115,7 +14114,7 @@
       <c r="Q32" s="10"/>
       <c r="R32" s="10"/>
     </row>
-    <row r="33" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="33" spans="1:18" ht="15" customHeight="1">
       <c r="A33" s="70" t="s">
         <v>406</v>
       </c>
@@ -14240,7 +14239,7 @@
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
     </row>
-    <row r="36" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="36" spans="1:18" ht="15" customHeight="1">
       <c r="A36" s="71" t="s">
         <v>413</v>
       </c>
@@ -14283,7 +14282,7 @@
       <c r="Q36" s="10"/>
       <c r="R36" s="10"/>
     </row>
-    <row r="37" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="37" spans="1:18" ht="15" customHeight="1">
       <c r="A37" s="71" t="s">
         <v>415</v>
       </c>
@@ -14324,7 +14323,7 @@
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
     </row>
-    <row r="38" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="38" spans="1:18" ht="15" customHeight="1">
       <c r="A38" s="71" t="s">
         <v>418</v>
       </c>
@@ -14365,7 +14364,7 @@
       <c r="Q38" s="10"/>
       <c r="R38" s="10"/>
     </row>
-    <row r="39" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="39" spans="1:18" ht="15" customHeight="1">
       <c r="A39" s="71" t="s">
         <v>421</v>
       </c>
@@ -14408,7 +14407,7 @@
       </c>
       <c r="R39" s="10"/>
     </row>
-    <row r="40" spans="1:18" ht="15" hidden="1" customHeight="1">
+    <row r="40" spans="1:18" ht="15" customHeight="1">
       <c r="A40" s="71" t="s">
         <v>424</v>
       </c>
@@ -18128,13 +18127,7 @@
       <c r="R224" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Q40" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="CISU"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:Q40" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A2:A1048576">
     <cfRule type="duplicateValues" dxfId="49" priority="24"/>
   </conditionalFormatting>

</xml_diff>